<commit_message>
completed acceptance test plan for cross team activity
</commit_message>
<xml_diff>
--- a/etc/Acceptance Test Plan.xlsx
+++ b/etc/Acceptance Test Plan.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="56">
   <si>
     <t>Instructions</t>
   </si>
@@ -248,9 +248,6 @@
   <si>
     <t>Given I am logged in as admin when I navigate to view the statistics then I am redirected to the statistics page.
 Given I am logged in as a helper when I try to access the statistics page then the website should route me elsewhere.</t>
-  </si>
-  <si>
-    <t>The Forgot Password button has not been implemented yet.</t>
   </si>
   <si>
     <t>This story has not been implemented yet.</t>
@@ -4247,7 +4244,9 @@
       </c>
       <c r="C16" s="11"/>
       <c r="D16" s="2"/>
-      <c r="E16" s="11"/>
+      <c r="E16" s="11" t="s">
+        <v>13</v>
+      </c>
       <c r="F16" s="2"/>
       <c r="G16" s="12"/>
       <c r="H16" s="12"/>
@@ -4279,7 +4278,9 @@
       </c>
       <c r="C17" s="11"/>
       <c r="D17" s="2"/>
-      <c r="E17" s="11"/>
+      <c r="E17" s="11" t="s">
+        <v>13</v>
+      </c>
       <c r="F17" s="2"/>
       <c r="G17" s="12"/>
       <c r="H17" s="12"/>
@@ -4311,7 +4312,9 @@
       </c>
       <c r="C18" s="11"/>
       <c r="D18" s="2"/>
-      <c r="E18" s="11"/>
+      <c r="E18" s="11" t="s">
+        <v>13</v>
+      </c>
       <c r="F18" s="2"/>
       <c r="G18" s="12"/>
       <c r="H18" s="12"/>
@@ -4343,10 +4346,10 @@
       </c>
       <c r="C19" s="11"/>
       <c r="D19" s="2"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="17" t="s">
-        <v>55</v>
+      <c r="E19" s="11" t="s">
+        <v>13</v>
       </c>
+      <c r="F19" s="17"/>
       <c r="G19" s="12"/>
       <c r="H19" s="12"/>
       <c r="I19" s="12"/>
@@ -4377,7 +4380,9 @@
       </c>
       <c r="C20" s="11"/>
       <c r="D20" s="2"/>
-      <c r="E20" s="11"/>
+      <c r="E20" s="11" t="s">
+        <v>13</v>
+      </c>
       <c r="F20" s="2"/>
       <c r="G20" s="12"/>
       <c r="H20" s="12"/>
@@ -4411,7 +4416,7 @@
       <c r="D21" s="2"/>
       <c r="E21" s="19"/>
       <c r="F21" s="20" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G21" s="12"/>
       <c r="H21" s="12"/>

</xml_diff>